<commit_message>
Tablero Sorpresa 16/10: cuadre contra Agrupadas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SmQ59SXzFJRTF75F5XCdhw
</commit_message>
<xml_diff>
--- a/ateneo/historial/2026-10/libros_sorpresa/Libros_Sorpresa_ventas_por_local.xlsx
+++ b/ateneo/historial/2026-10/libros_sorpresa/Libros_Sorpresa_ventas_por_local.xlsx
@@ -1027,7 +1027,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Solo locales físicos · del 01/10 al 16/10/2026 · el 16/10 es parcial (el reporte se sacó ese mismo día) · fuente: Detalle Venta Artículo (sin Ventas Agrupadas para cuadrar)</t>
+          <t>Solo locales físicos · del 01/10 al 16/10/2026 · el 16/10 es parcial (el reporte se sacó ese mismo día) · fuente: Detalle Venta Artículo, cuadrado contra Ventas Proveedor Agrupadas (Agrupadas trae 2 u más: se sacó después, son ventas del 16/10)</t>
         </is>
       </c>
     </row>
@@ -15167,7 +15167,7 @@
       </c>
       <c r="B2" s="28" t="inlineStr">
         <is>
-          <t>s/d (no se pasó Ventas Agrupadas) (la repo de Sorpresa se pasó el 05/10)</t>
+          <t>No (la repo de Sorpresa se pasó el 05/10)</t>
         </is>
       </c>
       <c r="C2" s="17" t="n">

</xml_diff>